<commit_message>
docs: 비용산정 Option A/B 파일 분리
</commit_message>
<xml_diff>
--- a/content/02_리서치/2026-06-30_API비용산정_근거.xlsx
+++ b/content/02_리서치/2026-06-30_API비용산정_근거.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -62,11 +62,6 @@
       <name val="맑은 고딕"/>
       <b val="1"/>
       <color rgb="00C00000"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="맑은 고딕"/>
-      <color rgb="00666666"/>
       <sz val="10"/>
     </font>
     <font>
@@ -132,7 +127,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -152,19 +147,19 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -187,11 +182,6 @@
     </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -204,16 +194,16 @@
     <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -581,8 +571,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I46"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:H43"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -597,7 +587,7 @@
     <row r="1" ht="21" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>KX_A2 · 1개월 예상 비용 (청구용)</t>
+          <t>KX_A2 · 1개월 예상 비용 (청구용) — Claude Code Option A: Pro×6</t>
         </is>
       </c>
     </row>
@@ -608,7 +598,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="16.5" customHeight="1">
+    <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>환율 (KRW/USD)</t>
@@ -623,7 +613,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="16.5" customHeight="1">
+    <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>청구 기간</t>
@@ -642,7 +632,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="16.5" customHeight="1">
+    <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
           <t>항목</t>
@@ -676,7 +666,7 @@
       <c r="G8" s="6" t="inlineStr"/>
       <c r="H8" s="6" t="inlineStr"/>
     </row>
-    <row r="9" ht="16.5" customHeight="1">
+    <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Figma Professional (월간)</t>
@@ -692,7 +682,7 @@
         <f>B9*C9</f>
         <v/>
       </c>
-      <c r="E9" s="8">
+      <c r="E9" s="4">
         <f>D9*$B$4</f>
         <v/>
       </c>
@@ -702,7 +692,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="16.5" customHeight="1">
+    <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
           <t>Vercel</t>
@@ -714,7 +704,7 @@
       <c r="C10" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="D10" s="9" t="n">
+      <c r="D10" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E10" s="4" t="n">
@@ -726,7 +716,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="16.5" customHeight="1">
+    <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
           <t>Supabase Pro</t>
@@ -742,7 +732,7 @@
         <f>B11*C11</f>
         <v/>
       </c>
-      <c r="E11" s="8">
+      <c r="E11" s="4">
         <f>D11*$B$4</f>
         <v/>
       </c>
@@ -752,7 +742,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="16.5" customHeight="1">
+    <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
           <t>AWS (EC2·S3·RDS 예비 예산)</t>
@@ -768,7 +758,7 @@
         <f>B12*C12</f>
         <v/>
       </c>
-      <c r="E12" s="8">
+      <c r="E12" s="4">
         <f>D12*$B$4</f>
         <v/>
       </c>
@@ -778,10 +768,10 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="16.5" customHeight="1">
+    <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>[Option A] Claude Code Pro × 6명</t>
+          <t>Claude Code Pro × 6명</t>
         </is>
       </c>
       <c r="B13" s="5" t="n">
@@ -794,130 +784,126 @@
         <f>B13*C13</f>
         <v/>
       </c>
-      <c r="E13" s="8">
+      <c r="E13" s="4">
         <f>D13*$B$4</f>
         <v/>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>Pro $20/유저 — 기본 플랜</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="16.5" customHeight="1">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>[Option B] Claude Code Max×4 + Pro×2</t>
-        </is>
-      </c>
-      <c r="B14" s="10" t="inlineStr">
-        <is>
-          <t>Max×4+Pro×2</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>6명</t>
-        </is>
-      </c>
-      <c r="D14" s="9" t="n">
-        <v>440</v>
-      </c>
-      <c r="E14" s="8">
+          <t>Pro $20/유저</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>고정 소계</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="n"/>
+      <c r="C14" s="9" t="n"/>
+      <c r="D14" s="10">
+        <f>SUM(D9:D13)</f>
+        <v/>
+      </c>
+      <c r="E14" s="11">
         <f>D14*$B$4</f>
         <v/>
       </c>
-      <c r="F14" s="5" t="inlineStr">
-        <is>
-          <t>Max $100(BE2·FE1·UX1) + Pro $20(PM2) — 업그레이드 불가 시 권장</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="16.5" customHeight="1">
-      <c r="A15" s="11" t="inlineStr">
-        <is>
-          <t>고정 소계 (Option A 기준)</t>
-        </is>
-      </c>
-      <c r="B15" s="12" t="n"/>
-      <c r="C15" s="12" t="n"/>
-      <c r="D15" s="7">
-        <f>D9+D10+D11+D12+D13</f>
-        <v/>
-      </c>
-      <c r="E15" s="8">
-        <f>D15*$B$4</f>
-        <v/>
-      </c>
-      <c r="F15" s="13" t="inlineStr">
-        <is>
-          <t>※ Option B 기준: D열 합계 $515</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="16.5" customHeight="1">
-      <c r="A17" s="2" t="inlineStr">
+    </row>
+    <row r="16" ht="16.5" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>② 사용량 기반 API — 토큰 기반 (Claude Sonnet)</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="16.5" customHeight="1">
-      <c r="A18" s="6" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
         <is>
           <t>항목</t>
         </is>
       </c>
-      <c r="B18" s="6" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>호출수</t>
         </is>
       </c>
-      <c r="C18" s="6" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>입력토큰/회</t>
         </is>
       </c>
-      <c r="D18" s="6" t="inlineStr">
+      <c r="D17" s="6" t="inlineStr">
         <is>
           <t>출력토큰/회</t>
         </is>
       </c>
-      <c r="E18" s="6" t="inlineStr">
+      <c r="E17" s="6" t="inlineStr">
         <is>
           <t>입력단가($/1M)</t>
         </is>
       </c>
-      <c r="F18" s="6" t="inlineStr">
+      <c r="F17" s="6" t="inlineStr">
         <is>
           <t>출력단가($/1M)</t>
         </is>
       </c>
-      <c r="G18" s="6" t="inlineStr">
+      <c r="G17" s="6" t="inlineStr">
         <is>
           <t>합계(USD)</t>
         </is>
       </c>
-      <c r="H18" s="6" t="inlineStr">
+      <c r="H17" s="6" t="inlineStr">
         <is>
           <t>합계(KRW)</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="16.5" customHeight="1">
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Claude Sonnet — 프롬프트 보조 (F001)</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>350</v>
+      </c>
+      <c r="C18" s="5" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D18" s="5" t="n">
+        <v>600</v>
+      </c>
+      <c r="E18" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F18" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="G18" s="7">
+        <f>B18*(C18*E18+D18*F18)/1000000</f>
+        <v/>
+      </c>
+      <c r="H18" s="4">
+        <f>G18*$B$4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Claude Sonnet — 프롬프트 보조 (F001)</t>
+          <t>Claude Sonnet — 역프롬프트 (F004, S등급)</t>
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>350</v>
+        <v>150</v>
       </c>
       <c r="C19" s="5" t="n">
-        <v>2000</v>
+        <v>2500</v>
       </c>
       <c r="D19" s="5" t="n">
-        <v>600</v>
+        <v>800</v>
       </c>
       <c r="E19" s="5" t="n">
         <v>3</v>
@@ -929,251 +915,244 @@
         <f>B19*(C19*E19+D19*F19)/1000000</f>
         <v/>
       </c>
-      <c r="H19" s="8">
+      <c r="H19" s="4">
         <f>G19*$B$4</f>
         <v/>
       </c>
-      <c r="I19" s="5" t="inlineStr">
-        <is>
-          <t>이미지 프롬프트 생성 보조</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="16.5" customHeight="1">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>Claude Sonnet — 역프롬프트 (F004, S등급)</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="n">
-        <v>150</v>
-      </c>
-      <c r="C20" s="5" t="n">
-        <v>2500</v>
-      </c>
-      <c r="D20" s="5" t="n">
-        <v>800</v>
-      </c>
-      <c r="E20" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="F20" s="5" t="n">
-        <v>15</v>
-      </c>
-      <c r="G20" s="7">
-        <f>B20*(C20*E20+D20*F20)/1000000</f>
-        <v/>
-      </c>
-      <c r="H20" s="8">
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>API 소계</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="n"/>
+      <c r="C20" s="9" t="n"/>
+      <c r="D20" s="9" t="n"/>
+      <c r="E20" s="9" t="n"/>
+      <c r="F20" s="9" t="n"/>
+      <c r="G20" s="10">
+        <f>SUM(G18:G19)</f>
+        <v/>
+      </c>
+      <c r="H20" s="11">
         <f>G20*$B$4</f>
         <v/>
       </c>
-      <c r="I20" s="5" t="inlineStr">
-        <is>
-          <t>역프롬프트 분석 (S등급 도전)</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="16.5" customHeight="1">
-      <c r="A21" s="11" t="inlineStr">
-        <is>
-          <t>API 소계</t>
-        </is>
-      </c>
-      <c r="B21" s="12" t="n"/>
-      <c r="C21" s="12" t="n"/>
-      <c r="D21" s="12" t="n"/>
-      <c r="E21" s="12" t="n"/>
-      <c r="F21" s="12" t="n"/>
-      <c r="G21" s="7">
-        <f>SUM(G19:G20)</f>
-        <v/>
-      </c>
-      <c r="H21" s="8">
-        <f>G21*$B$4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23" ht="16.5" customHeight="1">
-      <c r="A23" s="2" t="inlineStr">
+    </row>
+    <row r="22" ht="16.5" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>③ 사용량 기반 — 이미지 생성 (GPT Image 2, quality: medium)</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="16.5" customHeight="1">
-      <c r="A24" s="6" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
         <is>
           <t>항목</t>
         </is>
       </c>
-      <c r="B24" s="6" t="inlineStr">
+      <c r="B23" s="6" t="inlineStr">
         <is>
           <t>이미지 수</t>
         </is>
       </c>
-      <c r="C24" s="6" t="inlineStr">
+      <c r="C23" s="6" t="inlineStr">
         <is>
           <t>단가/장(USD)</t>
         </is>
       </c>
-      <c r="D24" s="6" t="inlineStr">
+      <c r="D23" s="6" t="inlineStr">
         <is>
           <t>합계(USD)</t>
         </is>
       </c>
-      <c r="E24" s="6" t="inlineStr">
+      <c r="E23" s="6" t="inlineStr">
         <is>
           <t>합계(KRW)</t>
         </is>
       </c>
-      <c r="F24" s="6" t="inlineStr">
+      <c r="F23" s="6" t="inlineStr">
         <is>
           <t>비고</t>
         </is>
       </c>
-      <c r="G24" s="6" t="inlineStr"/>
-      <c r="H24" s="6" t="inlineStr"/>
-    </row>
-    <row r="25" ht="16.5" customHeight="1">
-      <c r="A25" s="3" t="inlineStr">
+      <c r="G23" s="6" t="inlineStr"/>
+      <c r="H23" s="6" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
         <is>
           <t>GPT Image 2 medium — 단일 이미지 (F001)</t>
         </is>
       </c>
-      <c r="B25" s="5" t="n">
+      <c r="B24" s="5" t="n">
         <v>120</v>
       </c>
-      <c r="C25" s="5" t="n">
+      <c r="C24" s="5" t="n">
         <v>0.042</v>
       </c>
-      <c r="D25" s="7">
-        <f>B25*C25</f>
-        <v/>
-      </c>
-      <c r="E25" s="8">
-        <f>D25*$B$4</f>
-        <v/>
-      </c>
-      <c r="F25" s="5" t="inlineStr">
+      <c r="D24" s="7">
+        <f>B24*C24</f>
+        <v/>
+      </c>
+      <c r="E24" s="4">
+        <f>D24*$B$4</f>
+        <v/>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
         <is>
           <t>이미지 생성 테스트+데모</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="16.5" customHeight="1">
-      <c r="A26" s="14" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="12" t="inlineStr">
         <is>
           <t>[B팀 제공] 9그리드 스토리보드</t>
         </is>
       </c>
-      <c r="B26" s="15" t="n">
+      <c r="B25" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="C26" s="15" t="n">
+      <c r="C25" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="D26" s="16" t="n">
+      <c r="D25" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="E26" s="17" t="n">
+      <c r="E25" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="F26" s="15" t="inlineStr">
+      <c r="F25" s="13" t="inlineStr">
         <is>
           <t>B팀에서 생성 제공 → A2팀 비용 없음</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="16.5" customHeight="1">
-      <c r="A27" s="11" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr">
         <is>
           <t>이미지 소계</t>
         </is>
       </c>
-      <c r="B27" s="12" t="n"/>
-      <c r="C27" s="12" t="n"/>
-      <c r="D27" s="7">
-        <f>D25</f>
-        <v/>
-      </c>
-      <c r="E27" s="8">
-        <f>D27*$B$4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29" ht="16.5" customHeight="1">
-      <c r="A29" s="2" t="inlineStr">
+      <c r="B26" s="9" t="n"/>
+      <c r="C26" s="9" t="n"/>
+      <c r="D26" s="10">
+        <f>D24</f>
+        <v/>
+      </c>
+      <c r="E26" s="11">
+        <f>D26*$B$4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" ht="16.5" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>④ 사용량 기반 — 영상 생성 (fal.ai / 1세트 = 1클립)</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="16.5" customHeight="1">
-      <c r="A30" s="18" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  ℹ  흐름: [B팀] 9그리드 스토리보드 + shot1~9 프롬프트 제공  →  [A2팀] 영상 생성 API  →  클립 1개 출력</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="16.5" customHeight="1">
-      <c r="A31" s="6" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
         <is>
           <t>항목</t>
         </is>
       </c>
-      <c r="B31" s="6" t="inlineStr">
+      <c r="B30" s="6" t="inlineStr">
         <is>
           <t>단가($/초)</t>
         </is>
       </c>
-      <c r="C31" s="6" t="inlineStr">
+      <c r="C30" s="6" t="inlineStr">
         <is>
           <t>세트 수</t>
         </is>
       </c>
-      <c r="D31" s="6" t="inlineStr">
+      <c r="D30" s="6" t="inlineStr">
         <is>
           <t>초/클립</t>
         </is>
       </c>
-      <c r="E31" s="6" t="inlineStr">
+      <c r="E30" s="6" t="inlineStr">
         <is>
           <t>총 초</t>
         </is>
       </c>
-      <c r="F31" s="6" t="inlineStr">
+      <c r="F30" s="6" t="inlineStr">
         <is>
           <t>합계(USD)</t>
         </is>
       </c>
-      <c r="G31" s="6" t="inlineStr">
+      <c r="G30" s="6" t="inlineStr">
         <is>
           <t>합계(KRW)</t>
         </is>
       </c>
-      <c r="H31" s="6" t="inlineStr">
+      <c r="H30" s="6" t="inlineStr">
         <is>
           <t>비고</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="16.5" customHeight="1">
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>fal.ai Kling — 개발 테스트 (5초/클립)</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="C31" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="D31" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="E31" s="5">
+        <f>C31*D31</f>
+        <v/>
+      </c>
+      <c r="F31" s="7">
+        <f>B31*E31</f>
+        <v/>
+      </c>
+      <c r="G31" s="4">
+        <f>F31*$B$4</f>
+        <v/>
+      </c>
+      <c r="H31" s="5" t="inlineStr">
+        <is>
+          <t>주 2회×4주 / 3~5초 상한 기준</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>fal.ai Kling — 개발 테스트 (5초/클립)</t>
+          <t>fal.ai Seedance 2.0 — 중간점검 (5초/클립)</t>
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>0.11</v>
+        <v>0.3034</v>
       </c>
       <c r="C32" s="5" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="D32" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="E32" s="12">
+      <c r="E32" s="5">
         <f>C32*D32</f>
         <v/>
       </c>
@@ -1181,32 +1160,32 @@
         <f>B32*E32</f>
         <v/>
       </c>
-      <c r="G32" s="8">
+      <c r="G32" s="4">
         <f>F32*$B$4</f>
         <v/>
       </c>
       <c r="H32" s="5" t="inlineStr">
         <is>
-          <t>주 2회×4주 / 3~5초 상한 기준</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="16.5" customHeight="1">
+          <t>2주차 중간점검 데모 / 720p standard</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>fal.ai Seedance 2.0 — 중간점검 (5초/클립)</t>
+          <t>fal.ai Seedance 2.0 — 최종 출력 (15초/클립, 최대 길이)</t>
         </is>
       </c>
       <c r="B33" s="5" t="n">
         <v>0.3034</v>
       </c>
       <c r="C33" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D33" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="E33" s="12">
+        <v>15</v>
+      </c>
+      <c r="E33" s="5">
         <f>C33*D33</f>
         <v/>
       </c>
@@ -1214,235 +1193,167 @@
         <f>B33*E33</f>
         <v/>
       </c>
-      <c r="G33" s="8">
+      <c r="G33" s="4">
         <f>F33*$B$4</f>
         <v/>
       </c>
       <c r="H33" s="5" t="inlineStr">
         <is>
-          <t>2주차 중간점검 데모 / 720p standard</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="16.5" customHeight="1">
-      <c r="A34" s="3" t="inlineStr">
-        <is>
-          <t>fal.ai Seedance 2.0 — 최종 출력 (15초/클립, 최대 길이)</t>
-        </is>
-      </c>
-      <c r="B34" s="5" t="n">
-        <v>0.3034</v>
-      </c>
-      <c r="C34" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D34" s="5" t="n">
-        <v>15</v>
-      </c>
-      <c r="E34" s="12">
-        <f>C34*D34</f>
-        <v/>
-      </c>
-      <c r="F34" s="7">
-        <f>B34*E34</f>
-        <v/>
-      </c>
-      <c r="G34" s="8">
+          <t>4주차 최종 발표 2세트 / 720p / 음성 포함</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="inlineStr">
+        <is>
+          <t>영상 소계</t>
+        </is>
+      </c>
+      <c r="B34" s="9" t="n"/>
+      <c r="C34" s="9" t="n"/>
+      <c r="D34" s="9" t="n"/>
+      <c r="E34" s="9" t="n"/>
+      <c r="F34" s="10">
+        <f>SUM(F31:F33)</f>
+        <v/>
+      </c>
+      <c r="G34" s="11">
         <f>F34*$B$4</f>
         <v/>
       </c>
-      <c r="H34" s="5" t="inlineStr">
-        <is>
-          <t>4주차 최종 발표 2세트 / 720p / 음성 포함</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="16.5" customHeight="1">
-      <c r="A35" s="11" t="inlineStr">
-        <is>
-          <t>영상 소계</t>
-        </is>
-      </c>
-      <c r="B35" s="12" t="n"/>
-      <c r="C35" s="12" t="n"/>
-      <c r="D35" s="12" t="n"/>
-      <c r="E35" s="12" t="n"/>
-      <c r="F35" s="7">
-        <f>SUM(F32:F34)</f>
-        <v/>
-      </c>
-      <c r="G35" s="8">
-        <f>F35*$B$4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36" ht="16.5" customHeight="1">
-      <c r="A36" s="19" t="inlineStr">
+    </row>
+    <row r="35">
+      <c r="A35" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">  ★ fal.ai Hard Limit 권장 $50 설정 (Billing &gt; Spend Limit)</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="16.5" customHeight="1">
-      <c r="A38" s="2" t="inlineStr">
+    <row r="37" ht="16.5" customHeight="1">
+      <c r="A37" s="2" t="inlineStr">
         <is>
           <t>■ 요약</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="16.5" customHeight="1">
-      <c r="A39" s="6" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
         <is>
           <t>항목</t>
         </is>
       </c>
-      <c r="B39" s="6" t="inlineStr">
+      <c r="B38" s="6" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="C39" s="6" t="inlineStr">
+      <c r="C38" s="6" t="inlineStr">
         <is>
           <t>KRW</t>
         </is>
       </c>
-      <c r="D39" s="6" t="inlineStr"/>
-      <c r="E39" s="6" t="inlineStr"/>
-      <c r="F39" s="6" t="inlineStr"/>
-      <c r="G39" s="6" t="inlineStr"/>
-      <c r="H39" s="6" t="inlineStr"/>
-    </row>
-    <row r="40" ht="16.5" customHeight="1">
+      <c r="D38" s="6" t="inlineStr"/>
+      <c r="E38" s="6" t="inlineStr"/>
+      <c r="F38" s="6" t="inlineStr"/>
+      <c r="G38" s="6" t="inlineStr"/>
+      <c r="H38" s="6" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>① 고정 구독 소계</t>
+        </is>
+      </c>
+      <c r="B39" s="18">
+        <f>D14</f>
+        <v/>
+      </c>
+      <c r="C39" s="19">
+        <f>E14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>① 고정 구독 소계 (Option A)</t>
-        </is>
-      </c>
-      <c r="B40" s="20">
-        <f>D15</f>
-        <v/>
-      </c>
-      <c r="C40" s="21">
-        <f>E15</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41" ht="16.5" customHeight="1">
-      <c r="A41" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  └ Option B 기준 시</t>
-        </is>
-      </c>
-      <c r="B41" s="23">
-        <f>D9+D10+D11+D12+D14</f>
-        <v/>
-      </c>
-      <c r="C41" s="24">
+          <t>②③④ API/이미지/영상 소계 (B등급)</t>
+        </is>
+      </c>
+      <c r="B40" s="18">
+        <f>D26+F31+F32+G18</f>
+        <v/>
+      </c>
+      <c r="C40" s="19">
+        <f>B40*$B$4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>②③④ API/이미지/영상 소계 (S등급 도전)</t>
+        </is>
+      </c>
+      <c r="B41" s="18">
+        <f>D26+F31+F32+F33+G18+G19</f>
+        <v/>
+      </c>
+      <c r="C41" s="19">
         <f>B41*$B$4</f>
         <v/>
       </c>
     </row>
     <row r="42" ht="16.5" customHeight="1">
-      <c r="A42" s="3" t="inlineStr">
-        <is>
-          <t>②③④ API/이미지/영상 소계 (B등급)</t>
-        </is>
-      </c>
-      <c r="B42" s="20">
-        <f>D27+F32+F33+G19</f>
-        <v/>
-      </c>
-      <c r="C42" s="21">
+      <c r="A42" s="20" t="inlineStr">
+        <is>
+          <t>★ 총 합계 — B등급</t>
+        </is>
+      </c>
+      <c r="B42" s="21">
+        <f>D14+B40</f>
+        <v/>
+      </c>
+      <c r="C42" s="22">
         <f>B42*$B$4</f>
         <v/>
       </c>
-    </row>
-    <row r="43" ht="16.5" customHeight="1">
-      <c r="A43" s="3" t="inlineStr">
-        <is>
-          <t>②③④ API/이미지/영상 소계 (S등급 도전)</t>
-        </is>
-      </c>
-      <c r="B43" s="20">
-        <f>D27+F32+F33+F34+G19+G20</f>
-        <v/>
-      </c>
-      <c r="C43" s="21">
+      <c r="D42" s="23" t="n"/>
+      <c r="E42" s="23" t="n"/>
+      <c r="F42" s="23" t="n"/>
+      <c r="G42" s="23" t="n"/>
+      <c r="H42" s="23" t="n"/>
+    </row>
+    <row r="43" ht="18" customHeight="1">
+      <c r="A43" s="24" t="inlineStr">
+        <is>
+          <t>★ 총 합계 — S등급 (권장)</t>
+        </is>
+      </c>
+      <c r="B43" s="25">
+        <f>D14+B41</f>
+        <v/>
+      </c>
+      <c r="C43" s="26">
         <f>B43*$B$4</f>
         <v/>
       </c>
-    </row>
-    <row r="44" ht="16.5" customHeight="1">
-      <c r="A44" s="25" t="inlineStr">
-        <is>
-          <t>★ 총 합계 — B등급 · Option A</t>
-        </is>
-      </c>
-      <c r="B44" s="26">
-        <f>D15+D27+F32+F33+G19</f>
-        <v/>
-      </c>
-      <c r="C44" s="27">
-        <f>B44*$B$4</f>
-        <v/>
-      </c>
-      <c r="D44" s="28" t="n"/>
-      <c r="E44" s="28" t="n"/>
-      <c r="F44" s="28" t="n"/>
-      <c r="G44" s="28" t="n"/>
-      <c r="H44" s="28" t="n"/>
-    </row>
-    <row r="45" ht="18" customHeight="1">
-      <c r="A45" s="29" t="inlineStr">
-        <is>
-          <t>★ 총 합계 — S등급 · Option A (권장)</t>
-        </is>
-      </c>
-      <c r="B45" s="30">
-        <f>D15+B43</f>
-        <v/>
-      </c>
-      <c r="C45" s="31">
-        <f>B45*$B$4</f>
-        <v/>
-      </c>
-      <c r="D45" s="32" t="n"/>
-      <c r="E45" s="32" t="n"/>
-      <c r="F45" s="32" t="n"/>
-      <c r="G45" s="32" t="n"/>
-      <c r="H45" s="32" t="n"/>
-    </row>
-    <row r="46" ht="16.5" customHeight="1">
-      <c r="A46" s="25" t="inlineStr">
-        <is>
-          <t>★ 총 합계 — S등급 · Option B</t>
-        </is>
-      </c>
-      <c r="B46" s="26">
-        <f>D9+D10+D11+D12+D14+B43</f>
-        <v/>
-      </c>
-      <c r="C46" s="27">
-        <f>B46*$B$4</f>
-        <v/>
-      </c>
-      <c r="D46" s="28" t="n"/>
-      <c r="E46" s="28" t="n"/>
-      <c r="F46" s="28" t="n"/>
-      <c r="G46" s="28" t="n"/>
-      <c r="H46" s="28" t="n"/>
+      <c r="D43" s="27" t="n"/>
+      <c r="E43" s="27" t="n"/>
+      <c r="F43" s="27" t="n"/>
+      <c r="G43" s="27" t="n"/>
+      <c r="H43" s="27" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="9">
     <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A30:H30"/>
     <mergeCell ref="A29:H29"/>
     <mergeCell ref="A7:H7"/>
-    <mergeCell ref="A38:H38"/>
-    <mergeCell ref="A36:H36"/>
+    <mergeCell ref="A35:H35"/>
+    <mergeCell ref="A16:H16"/>
+    <mergeCell ref="A28:H28"/>
     <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A23:H23"/>
-    <mergeCell ref="A17:H17"/>
+    <mergeCell ref="A37:H37"/>
+    <mergeCell ref="A22:H22"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>